<commit_message>
results(concordance): 4-judge tables, dashboard, xlsx and band figures
fig_pipeline.png (1.2 MB) left out: over the 500 KB pre-commit limit; pdf/svg of the same figure are included.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/concordance_validation/CONCORDANCE_RESULTS.xlsx
+++ b/results/concordance_validation/CONCORDANCE_RESULTS.xlsx
@@ -455,12 +455,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bands (T1-T7)</t>
+          <t>Bands (T1-T7,T9)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DISJOINT |r| intervals: 0.1-0.2 / 0.2-0.3 / 0.3-0.4 / 0.4-0.5 / 0.5-0.6 / 0.6+. NOT cumulative.</t>
+          <t>DISJOINT |r| intervals 0.1-0.2 ... 0.6+. NOT cumulative.</t>
         </is>
       </c>
     </row>
@@ -472,7 +472,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>COARSE bands (0.1-0.3 / 0.3-0.5 / &gt;0.5) because the random arm has only 16 directions above |r| 0.3 and 1 above 0.4 -- fine bands make every Fisher test underpowered.</t>
+          <t>COARSE (0.1-0.3 / 0.3-0.5 / &gt;0.5): random has only 16 directions above |r| 0.3, so fine bands leave Fisher tests underpowered.</t>
         </is>
       </c>
     </row>
@@ -484,7 +484,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>metric % (n). '-' = that source has no features in that interval.</t>
+          <t>metric % (n). '-' = source has no features in that interval.</t>
         </is>
       </c>
     </row>
@@ -508,7 +508,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>All evaluations on held-out shards 281-311. Directions built and selected on shards &lt;281.</t>
+          <t>All evaluations on held-out shards 281-311. Directions built/selected on shards &lt;281.</t>
         </is>
       </c>
     </row>
@@ -520,67 +520,67 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>cross-chapter = published slate (distractors from a DIFFERENT ICD-9 chapter). same-chapter = hard negatives from the correct code's OWN chapter.</t>
+          <t>cross-chapter = published slate. same-chapter = hard negatives from the correct code's OWN ICD-9 chapter (primary condition).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Binary arm</t>
+          <t>GemmaScope pool</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PARTIAL removed from the option set, r-anchor dropped. 'PARTIAL-&gt;YES' = share of originally-PARTIAL features that become YES when forced to choose.</t>
+          <t>154 = the 113 tiered features plus a 41-feature expansion filling the 0.3-0.4 band, which the published tier rule leaves empty for every SAE.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Anchoring arm</t>
+          <t>Binary arm</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arm 0 = verbatim published prompt (states r). Arm 1 = identical minus the r sentence. DeepSeek only, r&gt;0.3 and above.</t>
+          <t>PARTIAL removed from the option set, r-anchor dropped.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Small-n caution</t>
+          <t>Anchoring arm (T9)</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Many fine cells have n&lt;=5 (keyword 0.1-0.2 n=2; probe 0.6+ n=2; PCA 0.4-0.5 n=1; gemmascope 0.5-0.6 n=4). Do not read those as estimates.</t>
+          <t>Arm 0 = published prompt (states r); Arm 1 = identical minus that sentence. Both judges, both domain SAEs, per-feature.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Known gaps</t>
+          <t>Population limits</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PCA has no same-chapter run. Anchoring is DeepSeek-only. Random: 16 directions above |r| 0.3 -- a census of 18,432 from ONE seed, not a sample.</t>
+          <t>NOT sampling limits -- complete populations: GemmaScope has 13 features above r&gt;0.4 and ZERO above 0.6 (of 16,384); random has 16 above |r| 0.3 and none above 0.433 (of 18,432); keyword has 39 directions total.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Files</t>
+          <t>Known gaps</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Per-table CSVs alongside this workbook in results/concordance_validation/.</t>
+          <t>PCA has no same-chapter run. All explanations are Sonnet-written (no second-explainer control).</t>
         </is>
       </c>
     </row>
@@ -1220,7 +1220,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1273,12 +1273,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>17 vs 34  -17 **</t>
+          <t>17 vs 34  -17 ** (n=100)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>85 vs 69  +16 ns</t>
+          <t>85 vs 69  +16 ns (n=136)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -1305,12 +1305,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>13 vs 35  -22 ***</t>
+          <t>13 vs 35  -22 *** (n=100)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>86 vs 81  +5 ns</t>
+          <t>86 vs 81  +5 ns (n=136)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1337,12 +1337,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10 vs 17  -7 ns</t>
+          <t>10 vs 17  -7 ns (n=100)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>76 vs 38  +38 **</t>
+          <t>76 vs 38  +38 ** (n=136)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1369,12 +1369,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>7 vs 18  -11 **</t>
+          <t>7 vs 18  -11 ** (n=100)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>75 vs 44  +31 *</t>
+          <t>75 vs 44  +31 * (n=136)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -1401,12 +1401,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>28 vs 34  -6 ns</t>
+          <t>28 vs 34  -6 ns (n=40)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>75 vs 69  +6 ns</t>
+          <t>75 vs 69  +6 ns (n=80)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1433,12 +1433,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>35 vs 35  +0 ns</t>
+          <t>35 vs 35  +0 ns (n=40)</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>86 vs 81  +5 ns</t>
+          <t>86 vs 81  +5 ns (n=80)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1465,12 +1465,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>8 vs 17  -9 ns</t>
+          <t>8 vs 17  -9 ns (n=40)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>66 vs 38  +28 *</t>
+          <t>66 vs 38  +28 * (n=80)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1497,12 +1497,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>22 vs 18  +4 ns</t>
+          <t>22 vs 18  +4 ns (n=40)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>72 vs 44  +28 *</t>
+          <t>72 vs 44  +28 * (n=80)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1529,12 +1529,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>15 vs 34  -19 ***</t>
+          <t>15 vs 34  -19 *** (n=100)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>88 vs 69  +19 *</t>
+          <t>88 vs 69  +19 * (n=137)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1561,12 +1561,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>23 vs 35  -12 *</t>
+          <t>23 vs 35  -12 * (n=100)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>90 vs 81  +9 ns</t>
+          <t>90 vs 81  +9 ns (n=137)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1593,12 +1593,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>8 vs 17  -9 *</t>
+          <t>8 vs 17  -9 * (n=100)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>73 vs 38  +35 **</t>
+          <t>73 vs 38  +35 ** (n=137)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1625,12 +1625,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8 vs 18  -10 *</t>
+          <t>8 vs 18  -10 * (n=100)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>76 vs 44  +32 *</t>
+          <t>76 vs 44  +32 * (n=137)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1642,7 +1642,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1657,12 +1657,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>2 vs 34  -32 ***</t>
+          <t>2 vs 34  -32 *** (n=100)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>67 vs 69  -2 ns</t>
+          <t>67 vs 69  -2 ns (n=9)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1674,7 +1674,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1689,12 +1689,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3 vs 35  -32 ***</t>
+          <t>3 vs 35  -32 *** (n=100)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>67 vs 81  -14 ns</t>
+          <t>67 vs 81  -14 ns (n=9)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1706,7 +1706,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1721,12 +1721,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0 vs 17  -17 ***</t>
+          <t>0 vs 17  -17 *** (n=100)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>78 vs 38  +40 ns</t>
+          <t>52 vs 38  +14 ns (n=50)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1738,7 +1738,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1753,12 +1753,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0 vs 18  -18 ***</t>
+          <t>0 vs 18  -18 *** (n=100)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>67 vs 44  +23 ns</t>
+          <t>46 vs 44  +2 ns (n=50)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1785,12 +1785,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>100 vs 34  +66 **</t>
+          <t>100 vs 34  +66 ** (n=6)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>96 vs 69  +27 *</t>
+          <t>96 vs 69  +27 * (n=26)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1817,12 +1817,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>100 vs 35  +65 **</t>
+          <t>100 vs 35  +65 ** (n=6)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>92 vs 81  +11 ns</t>
+          <t>92 vs 81  +11 ns (n=26)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1849,12 +1849,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>50 vs 17  +33 ns</t>
+          <t>50 vs 17  +33 ns (n=6)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>92 vs 38  +54 ***</t>
+          <t>92 vs 38  +54 *** (n=26)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1881,12 +1881,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>83 vs 18  +65 **</t>
+          <t>83 vs 18  +65 ** (n=6)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>96 vs 44  +52 ***</t>
+          <t>96 vs 44  +52 *** (n=26)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1913,12 +1913,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>28 vs 34  -6 ns</t>
+          <t>28 vs 34  -6 ns (n=18)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>29 vs 69  -40 *</t>
+          <t>29 vs 69  -40 * (n=21)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1945,12 +1945,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>28 vs 35  -7 ns</t>
+          <t>28 vs 35  -7 ns (n=18)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>38 vs 81  -43 *</t>
+          <t>38 vs 81  -43 * (n=21)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1977,12 +1977,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>22 vs 17  +5 ns</t>
+          <t>22 vs 17  +5 ns (n=18)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>24 vs 38  -14 ns</t>
+          <t>24 vs 38  -14 ns (n=21)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2009,12 +2009,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>28 vs 18  +10 ns</t>
+          <t>28 vs 18  +10 ns (n=18)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>38 vs 44  -6 ns</t>
+          <t>38 vs 44  -6 ns (n=21)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -2041,12 +2041,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>12 vs 34  -22 ns</t>
+          <t>12 vs 34  -22 ns (n=17)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>21 vs 69  -48 **</t>
+          <t>21 vs 69  -48 ** (n=24)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -2073,12 +2073,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>18 vs 35  -17 ns</t>
+          <t>18 vs 35  -17 ns (n=17)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>21 vs 81  -60 ***</t>
+          <t>21 vs 81  -60 *** (n=24)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -2105,12 +2105,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>12 vs 17  -5 ns</t>
+          <t>12 vs 17  -5 ns (n=17)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>17 vs 38  -21 ns</t>
+          <t>17 vs 38  -21 ns (n=24)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -2137,15 +2137,79 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>18 vs 18  +0 ns</t>
+          <t>18 vs 18  +0 ns (n=17)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>17 vs 44  -27 ns</t>
+          <t>17 vs 44  -27 ns (n=24)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>PCA (35)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>cross-chapter</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>15 vs 34  -19 * (n=34)</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>100 vs 69  +31 ns (n=1)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>PCA (35)</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>cross-chapter</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>12 vs 35  -23 ** (n=34)</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>100 vs 81  +19 ns (n=1)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>–</t>
         </is>
@@ -2162,212 +2226,480 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>prompt</t>
+          <t>Source</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>judge</t>
+          <t>Judge</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>band</t>
+          <t>Prompt</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>0.1-0.2</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>exact_YES</t>
+          <t>0.2-0.3</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>YES_PARTIAL</t>
+          <t>0.3-0.4</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>hit1</t>
+          <t>0.4-0.5</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>0.5-0.6</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>0.6+</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>anchored-YES retained</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>UNKNOWN %</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>SAE jumprelu (380)</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>anchored (r stated)</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>deepseek-v3</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>r&gt;0.3</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>280</v>
-      </c>
-      <c r="E2" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="F2" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0 (80)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>0 (20)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>18 (136)</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>30 (84)</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>60 (60)</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>anchored (r stated)</t>
+          <t>SAE jumprelu (380)</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>deepseek-v3</t>
+          <t>Sonnet</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>r&gt;0.4</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>280</v>
-      </c>
-      <c r="E3" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="F3" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="G3" t="inlineStr"/>
+          <t>de-anchored (no r)</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0 (80)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0 (20)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>18 (136)</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>30 (84)</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>62 (60)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>88%</t>
+        </is>
+      </c>
+      <c r="K3" t="n">
+        <v>3.4</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>SAE jumprelu (380)</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>anchored (r stated)</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>deepseek-v3</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>r&gt;0.5</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>144</v>
-      </c>
-      <c r="E4" t="n">
-        <v>48.6</v>
-      </c>
-      <c r="F4" t="n">
-        <v>100</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0 (80)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0 (20)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>18 (136)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>30 (84)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>60 (60)</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>SAE jumprelu (380)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>de-anchored (no r)</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>deepseek-v3</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>r&gt;0.3</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>280</v>
-      </c>
-      <c r="E5" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="F5" t="n">
-        <v>98.2</v>
-      </c>
-      <c r="G5" t="n">
-        <v>83.59999999999999</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0 (80)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0 (20)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>9 (136)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>11 (84)</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>35 (60)</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>45%</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>de-anchored (no r)</t>
+          <t>SAE vanilla (380)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>deepseek-v3</t>
+          <t>Sonnet</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>r&gt;0.4</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>280</v>
-      </c>
-      <c r="E6" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="F6" t="n">
-        <v>98.2</v>
-      </c>
-      <c r="G6" t="n">
-        <v>83.59999999999999</v>
-      </c>
+          <t>anchored (r stated)</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0 (86)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0 (14)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>15 (137)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>33 (70)</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>60 (73)</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>SAE vanilla (380)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sonnet</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>de-anchored (no r)</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>deepseek-v3</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>r&gt;0.5</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>144</v>
-      </c>
-      <c r="E7" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="F7" t="n">
-        <v>99.3</v>
-      </c>
-      <c r="G7" t="n">
-        <v>90.3</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>1 (86)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>0 (14)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>18 (137)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>26 (70)</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>59 (73)</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>83%</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SAE vanilla (380)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>anchored (r stated)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0 (86)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0 (14)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>15 (137)</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>33 (70)</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>60 (73)</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SAE vanilla (380)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>de-anchored (no r)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0 (86)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0 (14)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2 (137)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>13 (70)</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>29 (73)</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>35%</t>
+        </is>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -5337,7 +5669,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -5362,7 +5694,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>5 (41)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -5384,7 +5716,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -5409,7 +5741,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>5 (41)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -6291,7 +6623,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -6316,7 +6648,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>88 (41)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -6338,7 +6670,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -6363,7 +6695,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>95 (41)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -7245,7 +7577,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -7270,7 +7602,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>7 (41)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -7292,7 +7624,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -7317,7 +7649,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>5 (41)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -8199,7 +8531,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -8246,7 +8578,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9106,7 +9438,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9131,7 +9463,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>46 (41)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -9153,7 +9485,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -9178,7 +9510,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>41 (41)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -9919,7 +10251,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -9966,7 +10298,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -10826,7 +11158,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -10851,7 +11183,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>41 (41)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -10873,7 +11205,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SAE gemmascope (113)</t>
+          <t>SAE gemmascope (154)</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -10898,7 +11230,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>–</t>
+          <t>37 (41)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">

</xml_diff>